<commit_message>
Added low side fet diode
</commit_message>
<xml_diff>
--- a/projects/LTC7890_Buck/LTC7890_BOM.xlsx
+++ b/projects/LTC7890_Buck/LTC7890_BOM.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\UWRT\MarsRoverElectricalKiCad\projects\LTC7890_Buck\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{905A86F6-F0B7-4DC8-AD46-A896F5A138AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CA24CE4-5C3D-4702-86D2-0BCC7416AB73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{49714629-2E5D-47B8-A555-D616FDA96D84}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="127">
   <si>
     <t>Capacitor In</t>
   </si>
@@ -411,6 +411,12 @@
   </si>
   <si>
     <t>https://www.mouser.ca/ProductDetail/Samsung-Electro-Mechanics/CL32B475KCJZ4NE</t>
+  </si>
+  <si>
+    <t>V3PM10-M3/H</t>
+  </si>
+  <si>
+    <t>https://www.mouser.ca/ProductDetail/Vishay-Semiconductors/V3PM10-M3-H</t>
   </si>
 </sst>
 </file>
@@ -784,7 +790,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05E459BF-586A-4F4B-931A-B6F36BAD946F}">
-  <dimension ref="A1:U56"/>
+  <dimension ref="A1:U57"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21.6328125" customWidth="1"/>
@@ -1017,7 +1023,7 @@
         <v>0.32</v>
       </c>
       <c r="E14" s="1">
-        <f t="shared" ref="E14:E33" si="2">IF(COUNT(C14:D14)=2,D14*C14*IF(ISNUMBER(SEARCH("lcsc", F14)), U$2, 1),"")</f>
+        <f t="shared" ref="E14:E32" si="2">IF(COUNT(C14:D14)=2,D14*C14*IF(ISNUMBER(SEARCH("lcsc", F14)), U$2, 1),"")</f>
         <v>2.6304000000000001E-2</v>
       </c>
       <c r="F14" t="s">
@@ -1342,72 +1348,66 @@
     </row>
     <row r="32" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>104</v>
-      </c>
-      <c r="B32" t="s">
-        <v>10</v>
+        <v>125</v>
       </c>
       <c r="C32">
-        <v>0.1</v>
+        <v>2</v>
       </c>
       <c r="D32" s="1">
-        <v>0.71</v>
+        <v>0.53</v>
       </c>
       <c r="E32" s="1">
         <f t="shared" si="2"/>
-        <v>9.7269999999999995E-2</v>
+        <v>1.06</v>
       </c>
       <c r="F32" t="s">
-        <v>103</v>
-      </c>
-      <c r="Q32" t="s">
-        <v>38</v>
+        <v>126</v>
       </c>
     </row>
     <row r="33" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
+        <v>104</v>
+      </c>
+      <c r="B33" t="s">
+        <v>10</v>
+      </c>
+      <c r="C33">
+        <v>0.1</v>
+      </c>
+      <c r="D33" s="1">
+        <v>0.71</v>
+      </c>
+      <c r="E33" s="1">
+        <f>IF(COUNT(C33:D33)=2,D33*C33*IF(ISNUMBER(SEARCH("lcsc", F33)), U$2, 1),"")</f>
+        <v>9.7269999999999995E-2</v>
+      </c>
+      <c r="F33" t="s">
+        <v>103</v>
+      </c>
+      <c r="Q33" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
         <v>117</v>
       </c>
-      <c r="B33" t="str">
+      <c r="B34" t="str">
         <f>TEXT("1", "#")</f>
         <v>1</v>
       </c>
-      <c r="C33">
-        <v>0.04</v>
-      </c>
-      <c r="D33" s="1">
-        <v>0.34</v>
-      </c>
-      <c r="E33" s="1">
-        <f t="shared" si="2"/>
-        <v>1.8632000000000003E-2</v>
-      </c>
-      <c r="F33" t="s">
-        <v>118</v>
-      </c>
-      <c r="Q33" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
-        <v>85</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>86</v>
-      </c>
       <c r="C34">
         <v>0.04</v>
       </c>
       <c r="D34" s="1">
-        <v>0.12</v>
+        <v>0.34</v>
       </c>
       <c r="E34" s="1">
-        <f t="shared" ref="E34:E45" si="3">IF(COUNT(C34:D34)=2,D34*C34*IF(ISNUMBER(SEARCH("lcsc", F34)), U$2, 1),"")</f>
-        <v>6.5760000000000002E-3</v>
+        <f>IF(COUNT(C34:D34)=2,D34*C34*IF(ISNUMBER(SEARCH("lcsc", F34)), U$2, 1),"")</f>
+        <v>1.8632000000000003E-2</v>
       </c>
       <c r="F34" t="s">
-        <v>87</v>
+        <v>118</v>
       </c>
       <c r="Q34" t="s">
         <v>116</v>
@@ -1415,101 +1415,101 @@
     </row>
     <row r="35" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>66</v>
-      </c>
-      <c r="B35" t="s">
-        <v>13</v>
-      </c>
-      <c r="C35" t="s">
-        <v>51</v>
-      </c>
-      <c r="E35" s="1" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+        <v>85</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C35">
+        <v>0.04</v>
+      </c>
+      <c r="D35" s="1">
+        <v>0.12</v>
+      </c>
+      <c r="E35" s="1">
+        <f>IF(COUNT(C35:D35)=2,D35*C35*IF(ISNUMBER(SEARCH("lcsc", F35)), U$2, 1),"")</f>
+        <v>6.5760000000000002E-3</v>
+      </c>
+      <c r="F35" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q35" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>93</v>
+        <v>66</v>
       </c>
       <c r="B36" t="s">
-        <v>94</v>
-      </c>
-      <c r="C36">
-        <v>0.04</v>
-      </c>
-      <c r="D36" s="1">
-        <v>0.3</v>
-      </c>
-      <c r="E36" s="1">
-        <f t="shared" si="3"/>
-        <v>1.6440000000000003E-2</v>
-      </c>
-      <c r="F36" t="s">
-        <v>95</v>
-      </c>
-      <c r="Q36" t="s">
-        <v>72</v>
+        <v>13</v>
+      </c>
+      <c r="C36" t="s">
+        <v>51</v>
+      </c>
+      <c r="E36" s="1" t="str">
+        <f>IF(COUNT(C36:D36)=2,D36*C36*IF(ISNUMBER(SEARCH("lcsc", F36)), U$2, 1),"")</f>
+        <v/>
       </c>
     </row>
     <row r="37" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>44</v>
+        <v>93</v>
       </c>
       <c r="B37" t="s">
-        <v>45</v>
-      </c>
-      <c r="C37" t="s">
-        <v>29</v>
-      </c>
-      <c r="E37" s="1" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+        <v>94</v>
+      </c>
+      <c r="C37">
+        <v>0.04</v>
+      </c>
+      <c r="D37" s="1">
+        <v>0.3</v>
+      </c>
+      <c r="E37" s="1">
+        <f>IF(COUNT(C37:D37)=2,D37*C37*IF(ISNUMBER(SEARCH("lcsc", F37)), U$2, 1),"")</f>
+        <v>1.6440000000000003E-2</v>
+      </c>
+      <c r="F37" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q37" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="38" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B38" t="s">
-        <v>20</v>
-      </c>
-      <c r="C38">
-        <v>0.02</v>
-      </c>
-      <c r="D38" s="1">
-        <v>0.55000000000000004</v>
-      </c>
-      <c r="E38" s="1">
-        <f t="shared" si="3"/>
-        <v>1.5070000000000004E-2</v>
-      </c>
-      <c r="F38" t="s">
-        <v>43</v>
-      </c>
-      <c r="Q38" t="s">
-        <v>36</v>
+        <v>45</v>
+      </c>
+      <c r="C38" t="s">
+        <v>29</v>
+      </c>
+      <c r="E38" s="1" t="str">
+        <f>IF(COUNT(C38:D38)=2,D38*C38*IF(ISNUMBER(SEARCH("lcsc", F38)), U$2, 1),"")</f>
+        <v/>
       </c>
     </row>
     <row r="39" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>96</v>
+        <v>47</v>
       </c>
       <c r="B39" t="s">
-        <v>97</v>
+        <v>20</v>
       </c>
       <c r="C39">
         <v>0.02</v>
       </c>
       <c r="D39" s="1">
-        <v>0.52</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="E39" s="1">
-        <f t="shared" si="3"/>
-        <v>1.4248000000000002E-2</v>
+        <f>IF(COUNT(C39:D39)=2,D39*C39*IF(ISNUMBER(SEARCH("lcsc", F39)), U$2, 1),"")</f>
+        <v>1.5070000000000004E-2</v>
       </c>
       <c r="F39" t="s">
-        <v>98</v>
+        <v>43</v>
       </c>
       <c r="Q39" t="s">
         <v>36</v>
@@ -1517,23 +1517,23 @@
     </row>
     <row r="40" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B40" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C40">
         <v>0.02</v>
       </c>
       <c r="D40" s="1">
-        <v>0.51</v>
+        <v>0.52</v>
       </c>
       <c r="E40" s="1">
-        <f t="shared" si="3"/>
-        <v>1.3974000000000002E-2</v>
+        <f>IF(COUNT(C40:D40)=2,D40*C40*IF(ISNUMBER(SEARCH("lcsc", F40)), U$2, 1),"")</f>
+        <v>1.4248000000000002E-2</v>
       </c>
       <c r="F40" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="Q40" t="s">
         <v>36</v>
@@ -1541,256 +1541,280 @@
     </row>
     <row r="41" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>49</v>
+        <v>99</v>
+      </c>
+      <c r="B41" t="s">
+        <v>100</v>
       </c>
       <c r="C41">
-        <v>1</v>
+        <v>0.02</v>
       </c>
       <c r="D41" s="1">
-        <v>0.23</v>
+        <v>0.51</v>
       </c>
       <c r="E41" s="1">
-        <f t="shared" si="3"/>
-        <v>0.23</v>
+        <f>IF(COUNT(C41:D41)=2,D41*C41*IF(ISNUMBER(SEARCH("lcsc", F41)), U$2, 1),"")</f>
+        <v>1.3974000000000002E-2</v>
       </c>
       <c r="F41" t="s">
-        <v>50</v>
+        <v>101</v>
+      </c>
+      <c r="Q41" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="42" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>27</v>
-      </c>
-      <c r="B42" t="s">
-        <v>28</v>
+        <v>49</v>
       </c>
       <c r="C42">
-        <v>0.06</v>
+        <v>1</v>
       </c>
       <c r="D42" s="1">
-        <v>0.52</v>
+        <v>0.23</v>
       </c>
       <c r="E42" s="1">
-        <f t="shared" si="3"/>
-        <v>4.2744000000000004E-2</v>
+        <f>IF(COUNT(C42:D42)=2,D42*C42*IF(ISNUMBER(SEARCH("lcsc", F42)), U$2, 1),"")</f>
+        <v>0.23</v>
       </c>
       <c r="F42" t="s">
-        <v>40</v>
-      </c>
-      <c r="Q42" t="s">
-        <v>88</v>
+        <v>50</v>
       </c>
     </row>
     <row r="43" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>53</v>
+        <v>27</v>
+      </c>
+      <c r="B43" t="s">
+        <v>28</v>
       </c>
       <c r="C43">
-        <v>0.8</v>
+        <v>0.06</v>
       </c>
       <c r="D43" s="1">
-        <v>0.39</v>
+        <v>0.52</v>
       </c>
       <c r="E43" s="1">
-        <f t="shared" si="3"/>
-        <v>0.4274400000000001</v>
+        <f>IF(COUNT(C43:D43)=2,D43*C43*IF(ISNUMBER(SEARCH("lcsc", F43)), U$2, 1),"")</f>
+        <v>4.2744000000000004E-2</v>
       </c>
       <c r="F43" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="Q43" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
     </row>
     <row r="44" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>73</v>
-      </c>
-      <c r="E44" s="1" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+        <v>53</v>
+      </c>
+      <c r="C44">
+        <v>0.8</v>
+      </c>
+      <c r="D44" s="1">
+        <v>0.39</v>
+      </c>
+      <c r="E44" s="1">
+        <f>IF(COUNT(C44:D44)=2,D44*C44*IF(ISNUMBER(SEARCH("lcsc", F44)), U$2, 1),"")</f>
+        <v>0.4274400000000001</v>
+      </c>
+      <c r="F44" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q44" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="45" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>21</v>
-      </c>
-      <c r="C45">
-        <v>1</v>
-      </c>
-      <c r="D45" s="1">
-        <v>0.67</v>
-      </c>
-      <c r="E45" s="1">
-        <f t="shared" si="3"/>
-        <v>0.91790000000000016</v>
-      </c>
-      <c r="F45" t="s">
-        <v>35</v>
+        <v>73</v>
+      </c>
+      <c r="E45" s="1" t="str">
+        <f>IF(COUNT(C45:D45)=2,D45*C45*IF(ISNUMBER(SEARCH("lcsc", F45)), U$2, 1),"")</f>
+        <v/>
       </c>
     </row>
     <row r="46" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>23</v>
-      </c>
-      <c r="B46" t="s">
-        <v>24</v>
-      </c>
-      <c r="C46" t="s">
-        <v>29</v>
+        <v>21</v>
+      </c>
+      <c r="C46">
+        <v>1</v>
+      </c>
+      <c r="D46" s="1">
+        <v>0.67</v>
+      </c>
+      <c r="E46" s="1">
+        <f>IF(COUNT(C46:D46)=2,D46*C46*IF(ISNUMBER(SEARCH("lcsc", F46)), U$2, 1),"")</f>
+        <v>0.91790000000000016</v>
+      </c>
+      <c r="F46" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="47" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B47" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C47" t="s">
-        <v>51</v>
-      </c>
-      <c r="E47" s="1" t="str">
-        <f>IF(COUNT(C47:D47)=2,D47*C47*IF(ISNUMBER(SEARCH("lcsc", F47)), U$2, 1),"")</f>
-        <v/>
+        <v>29</v>
       </c>
     </row>
     <row r="48" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
+        <v>27</v>
+      </c>
+      <c r="B48" t="s">
+        <v>28</v>
+      </c>
+      <c r="C48" t="s">
+        <v>51</v>
+      </c>
+      <c r="E48" s="1" t="str">
+        <f>IF(COUNT(C48:D48)=2,D48*C48*IF(ISNUMBER(SEARCH("lcsc", F48)), U$2, 1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
         <v>84</v>
       </c>
-      <c r="B48" t="str">
+      <c r="B49" t="str">
         <f>TEXT("10", "#")</f>
         <v>10</v>
       </c>
-      <c r="C48">
+      <c r="C49">
         <v>0.4</v>
       </c>
-      <c r="D48" s="1">
+      <c r="D49" s="1">
         <v>0.94</v>
       </c>
-      <c r="E48" s="1">
-        <f>IF(COUNT(C48:D48)=2,D48*C48*IF(ISNUMBER(SEARCH("lcsc", F48)), U$2, 1),"")</f>
+      <c r="E49" s="1">
+        <f>IF(COUNT(C49:D49)=2,D49*C49*IF(ISNUMBER(SEARCH("lcsc", F49)), U$2, 1),"")</f>
         <v>0.51512000000000002</v>
       </c>
-      <c r="F48" t="s">
+      <c r="F49" t="s">
         <v>79</v>
       </c>
-      <c r="Q48" t="s">
+      <c r="Q49" t="s">
         <v>80</v>
-      </c>
-    </row>
-    <row r="49" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A49" t="s">
-        <v>66</v>
-      </c>
-      <c r="B49" t="s">
-        <v>13</v>
-      </c>
-      <c r="C49" t="s">
-        <v>29</v>
-      </c>
-      <c r="E49" s="1" t="str">
-        <f>IF(COUNT(C49:D49)=2,D49*C49*IF(ISNUMBER(SEARCH("lcsc", F49)), U$2, 1),"")</f>
-        <v/>
       </c>
     </row>
     <row r="50" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>74</v>
+        <v>66</v>
+      </c>
+      <c r="B50" t="s">
+        <v>13</v>
+      </c>
+      <c r="C50" t="s">
+        <v>29</v>
+      </c>
+      <c r="E50" s="1" t="str">
+        <f>IF(COUNT(C50:D50)=2,D50*C50*IF(ISNUMBER(SEARCH("lcsc", F50)), U$2, 1),"")</f>
+        <v/>
       </c>
     </row>
     <row r="51" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>48</v>
-      </c>
-      <c r="C51">
-        <v>2</v>
-      </c>
-      <c r="D51" s="1">
-        <v>0.57999999999999996</v>
-      </c>
-      <c r="E51" s="1">
-        <f>IF(COUNT(C51:D51)=2,D51*C51*IF(ISNUMBER(SEARCH("lcsc", F51)), U$2, 1),"")</f>
-        <v>1.1599999999999999</v>
-      </c>
-      <c r="F51" t="s">
-        <v>92</v>
+        <v>74</v>
       </c>
     </row>
     <row r="52" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>30</v>
-      </c>
-      <c r="E52" s="1" t="str">
+        <v>48</v>
+      </c>
+      <c r="C52">
+        <v>2</v>
+      </c>
+      <c r="D52" s="1">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="E52" s="1">
         <f>IF(COUNT(C52:D52)=2,D52*C52*IF(ISNUMBER(SEARCH("lcsc", F52)), U$2, 1),"")</f>
-        <v/>
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="F52" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="53" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>75</v>
-      </c>
-      <c r="C53">
-        <v>1</v>
-      </c>
-      <c r="D53" s="1">
-        <v>0.47</v>
-      </c>
-      <c r="E53" s="1">
+        <v>30</v>
+      </c>
+      <c r="E53" s="1" t="str">
         <f>IF(COUNT(C53:D53)=2,D53*C53*IF(ISNUMBER(SEARCH("lcsc", F53)), U$2, 1),"")</f>
-        <v>0.64390000000000003</v>
-      </c>
-      <c r="F53" t="s">
-        <v>76</v>
+        <v/>
       </c>
     </row>
     <row r="54" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>32</v>
+        <v>75</v>
       </c>
       <c r="C54">
         <v>1</v>
       </c>
       <c r="D54" s="1">
-        <v>0.5</v>
+        <v>0.47</v>
       </c>
       <c r="E54" s="1">
         <f>IF(COUNT(C54:D54)=2,D54*C54*IF(ISNUMBER(SEARCH("lcsc", F54)), U$2, 1),"")</f>
-        <v>0.68500000000000005</v>
+        <v>0.64390000000000003</v>
       </c>
       <c r="F54" t="s">
-        <v>33</v>
+        <v>76</v>
       </c>
     </row>
     <row r="55" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C55">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="D55" s="1">
-        <v>1.27</v>
+        <v>0.5</v>
       </c>
       <c r="E55" s="1">
         <f>IF(COUNT(C55:D55)=2,D55*C55*IF(ISNUMBER(SEARCH("lcsc", F55)), U$2, 1),"")</f>
+        <v>0.68500000000000005</v>
+      </c>
+      <c r="F55" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="56" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
+        <v>31</v>
+      </c>
+      <c r="C56">
+        <v>0.4</v>
+      </c>
+      <c r="D56" s="1">
+        <v>1.27</v>
+      </c>
+      <c r="E56" s="1">
+        <f>IF(COUNT(C56:D56)=2,D56*C56*IF(ISNUMBER(SEARCH("lcsc", F56)), U$2, 1),"")</f>
         <v>0.69596000000000002</v>
       </c>
-      <c r="F55" t="s">
+      <c r="F56" t="s">
         <v>77</v>
       </c>
-      <c r="Q55" t="s">
+      <c r="Q56" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="56" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="D56" s="1" t="s">
+    <row r="57" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="D57" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="E56" s="1">
-        <f>SUM(E2:E55)</f>
-        <v>91.579988000000014</v>
+      <c r="E57" s="1">
+        <f>SUM(E2:E56)</f>
+        <v>92.639988000000017</v>
       </c>
     </row>
   </sheetData>

</xml_diff>